<commit_message>
Add final_url_path column to bulk upload for flexible URL construction - allows base URL + path combination
</commit_message>
<xml_diff>
--- a/bulk_upload_template.xlsx
+++ b/bulk_upload_template.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X4"/>
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -466,10 +466,11 @@
     <col width="34" customWidth="1" min="18" max="18"/>
     <col width="34" customWidth="1" min="19" max="19"/>
     <col width="32" customWidth="1" min="20" max="20"/>
-    <col width="29" customWidth="1" min="21" max="21"/>
-    <col width="50" customWidth="1" min="22" max="22"/>
-    <col width="37" customWidth="1" min="23" max="23"/>
-    <col width="23" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="50" customWidth="1" min="23" max="23"/>
+    <col width="37" customWidth="1" min="24" max="24"/>
+    <col width="23" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -580,15 +581,20 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
+          <t>final_url_path</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
           <t>keywords</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>headline_positions</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>description_positions</t>
         </is>
@@ -702,15 +708,20 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
+          <t>/services</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
           <t>PPCL services;professional services;consultation;expert PPCL</t>
         </is>
       </c>
-      <c r="W2" s="2" t="inlineStr">
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>1;2;3;4;5;6;7;8;9;10;11;12;13;14;15</t>
         </is>
       </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>1;2;3;4</t>
         </is>
@@ -819,20 +830,25 @@
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>https://ppcl.com/services</t>
+          <t>https://ppcl.com</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
+          <t>/consulting</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
           <t>PPCL experts;professional advice;guidance;trusted advisors</t>
         </is>
       </c>
-      <c r="W3" s="2" t="inlineStr">
+      <c r="X3" s="2" t="inlineStr">
         <is>
           <t>1;2;3;4;5;6;7;8;9;10;11;12;13;14;15</t>
         </is>
       </c>
-      <c r="X3" s="2" t="inlineStr">
+      <c r="Y3" s="2" t="inlineStr">
         <is>
           <t>1;2;3;4</t>
         </is>
@@ -941,20 +957,25 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>https://ppcl.com/consulting</t>
+          <t>https://ppcl.com</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
+          <t>/contact</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
           <t>PPCL consulting;expert advice;professional help;consulting services</t>
         </is>
       </c>
-      <c r="W4" s="2" t="inlineStr">
+      <c r="X4" s="2" t="inlineStr">
         <is>
           <t>1;2;3;4;5;6;7;8;9;10;11;12;13;14;15</t>
         </is>
       </c>
-      <c r="X4" s="2" t="inlineStr">
+      <c r="Y4" s="2" t="inlineStr">
         <is>
           <t>1;2;3;4</t>
         </is>
@@ -971,7 +992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1018,174 +1039,212 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>• final_url - Landing page URL</t>
+          <t>• final_url - Base landing page URL (e.g., https://example.com)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>• final_url_path - URL path to append (e.g., /services, /contact, /about)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>• keywords - Keywords separated by semicolons (e.g., 'keyword1;keyword2')</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>OPTIONAL COLUMNS:</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>• headline_positions - Headline positions separated by semicolons</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>• headline_positions - Headline positions separated by semicolons</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>• description_positions - Description positions separated by semicolons</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>IMPORTANT NOTES:</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>• Budget is set at campaign level (not in this file)</t>
+          <t>URL CONSTRUCTION:</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>• All rows go to one campaign (specified in the app)</t>
+          <t>• Final URL = final_url + final_url_path</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>• Keywords support match types: keyword (broad), 'keyword' (phrase), [keyword] (exact)</t>
+          <t>• Example: final_url='https://ppcl.com' + final_url_path='/services' = 'https://ppcl.com/services'</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>• Each row creates one ad</t>
+          <t>• If final_url_path is empty, only final_url is used</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>• Keywords are applied per ad group (uses first row's keywords)</t>
-        </is>
-      </c>
+      <c r="A19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>IMPORTANT NOTES:</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>EXAMPLE KEYWORDS:</t>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>• Budget is set at campaign level (not in this file)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>• Broad match: PPCL services</t>
+          <t>• All rows go to one campaign (specified in the app)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>• Phrase match: 'PPCL services'</t>
+          <t>• Keywords support match types: keyword (broad), 'keyword' (phrase), [keyword] (exact)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• Exact match: [PPCL services]</t>
+          <t>• Each row creates one ad</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>• Keywords are applied per ad group (uses first row's keywords)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>FILE FORMAT:</t>
-        </is>
-      </c>
+      <c r="A26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>• Save as .xlsx or .csv</t>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>EXAMPLE KEYWORDS:</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• UTF-8 encoding recommended</t>
+          <t>• Broad match: PPCL services</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>• Phrase match: 'PPCL services'</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>USAGE:</t>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>• Exact match: [PPCL services]</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>1. Fill in your data in the 'Bulk Upload Template' sheet</t>
-        </is>
-      </c>
+      <c r="A31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2. Save the file</t>
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>FILE FORMAT:</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>3. Upload in the app's Bulk Upload tab</t>
+          <t>• Save as .xlsx or .csv</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
+        <is>
+          <t>• UTF-8 encoding recommended</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>USAGE:</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>1. Fill in your data in the 'Bulk Upload Template' sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2. Save the file</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>3. Upload in the app's Bulk Upload tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>4. Set campaign name and monthly budget in the app</t>
         </is>

</xml_diff>

<commit_message>
Add Path 1 and Path 2 support for display URLs in bulk upload template and API
</commit_message>
<xml_diff>
--- a/bulk_upload_template.xlsx
+++ b/bulk_upload_template.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y4"/>
+  <dimension ref="A1:Z4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -467,10 +467,11 @@
     <col width="34" customWidth="1" min="19" max="19"/>
     <col width="32" customWidth="1" min="20" max="20"/>
     <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="50" customWidth="1" min="23" max="23"/>
-    <col width="37" customWidth="1" min="24" max="24"/>
-    <col width="23" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="7" customWidth="1" min="23" max="23"/>
+    <col width="50" customWidth="1" min="24" max="24"/>
+    <col width="37" customWidth="1" min="25" max="25"/>
+    <col width="23" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -581,20 +582,25 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>final_url_path</t>
+          <t>path1</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
+          <t>path2</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
           <t>keywords</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>headline_positions</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>description_positions</t>
         </is>
@@ -708,20 +714,21 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>/services</t>
-        </is>
-      </c>
-      <c r="W2" s="2" t="inlineStr">
+          <t>services</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>PPCL services;professional services;consultation;expert PPCL</t>
         </is>
       </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>1;2;3;4;5;6;7;8;9;10;11;12;13;14;15</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>1;2;3;4</t>
         </is>
@@ -835,20 +842,21 @@
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>/consulting</t>
-        </is>
-      </c>
-      <c r="W3" s="2" t="inlineStr">
+          <t>consulting</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr">
         <is>
           <t>PPCL experts;professional advice;guidance;trusted advisors</t>
         </is>
       </c>
-      <c r="X3" s="2" t="inlineStr">
+      <c r="Y3" s="2" t="inlineStr">
         <is>
           <t>1;2;3;4;5;6;7;8;9;10;11;12;13;14;15</t>
         </is>
       </c>
-      <c r="Y3" s="2" t="inlineStr">
+      <c r="Z3" s="2" t="inlineStr">
         <is>
           <t>1;2;3;4</t>
         </is>
@@ -962,20 +970,21 @@
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>/contact</t>
-        </is>
-      </c>
-      <c r="W4" s="2" t="inlineStr">
+          <t>contact</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr">
         <is>
           <t>PPCL consulting;expert advice;professional help;consulting services</t>
         </is>
       </c>
-      <c r="X4" s="2" t="inlineStr">
+      <c r="Y4" s="2" t="inlineStr">
         <is>
           <t>1;2;3;4;5;6;7;8;9;10;11;12;13;14;15</t>
         </is>
       </c>
-      <c r="Y4" s="2" t="inlineStr">
+      <c r="Z4" s="2" t="inlineStr">
         <is>
           <t>1;2;3;4</t>
         </is>
@@ -992,7 +1001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1046,205 +1055,219 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>• final_url_path - URL path to append (e.g., /services, /contact, /about)</t>
+          <t>• path1 - First display URL path (e.g., services, contact, about)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>• path2 - Second display URL path (optional, e.g., quote, info)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>• keywords - Keywords separated by semicolons (e.g., 'keyword1;keyword2')</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>OPTIONAL COLUMNS:</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>• headline_positions - Headline positions separated by semicolons</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>• headline_positions - Headline positions separated by semicolons</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>• description_positions - Description positions separated by semicolons</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>URL CONSTRUCTION:</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>• Final URL = final_url + final_url_path</t>
+          <t>URL CONSTRUCTION:</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>• Example: final_url='https://ppcl.com' + final_url_path='/services' = 'https://ppcl.com/services'</t>
+          <t>• Final URL = final_url (actual landing page)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>• If final_url_path is empty, only final_url is used</t>
+          <t>• Display URL = final_url + /path1 + /path2 (what users see in ads)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>• Example: final_url='https://ppcl.com' + path1='services' = display URL 'https://ppcl.com/services'</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>• Path1 and Path2 are for display only and don't affect the actual landing page</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>IMPORTANT NOTES:</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>• Budget is set at campaign level (not in this file)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>• All rows go to one campaign (specified in the app)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>• Keywords support match types: keyword (broad), 'keyword' (phrase), [keyword] (exact)</t>
+          <t>• Budget is set at campaign level (not in this file)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• Each row creates one ad</t>
+          <t>• All rows go to one campaign (specified in the app)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>• Keywords support match types: keyword (broad), 'keyword' (phrase), [keyword] (exact)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>• Each row creates one ad</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>• Keywords are applied per ad group (uses first row's keywords)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>EXAMPLE KEYWORDS:</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>• Broad match: PPCL services</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>• Phrase match: 'PPCL services'</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>• Broad match: PPCL services</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>• Phrase match: 'PPCL services'</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>• Exact match: [PPCL services]</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>FILE FORMAT:</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>• Save as .xlsx or .csv</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>• UTF-8 encoding recommended</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>USAGE:</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>1. Fill in your data in the 'Bulk Upload Template' sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2. Save the file</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>3. Upload in the app's Bulk Upload tab</t>
+          <t>1. Fill in your data in the 'Bulk Upload Template' sheet</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
+        <is>
+          <t>2. Save the file</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>3. Upload in the app's Bulk Upload tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>4. Set campaign name and monthly budget in the app</t>
         </is>

</xml_diff>